<commit_message>
Control for local co-occurrences The second version of stimuli after manual removal of collocations. Also adds the original cnt_zh.
</commit_message>
<xml_diff>
--- a/output/full_design_v1.xlsx
+++ b/output/full_design_v1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cmailcarletonca-my.sharepoint.com/personal/fengweiliu_cmail_carleton_ca/Documents/Bilingual_Semantics/Stimuli/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="122" documentId="11_A9F47193D29D5AB3B55B81AAC79DDC3817857819" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{212700BF-57EF-8B4D-A427-746894A2BF0B}"/>
+  <xr:revisionPtr revIDLastSave="123" documentId="11_A9F47193D29D5AB3B55B81AAC79DDC3817857819" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{631BD9BF-48B5-FE42-AFA9-C548EED9ED4A}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6540" uniqueCount="775">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6540" uniqueCount="776">
   <si>
     <t>stim_id</t>
   </si>
@@ -2350,6 +2350,9 @@
   </si>
   <si>
     <t>counterbalanced list id</t>
+  </si>
+  <si>
+    <t>x</t>
   </si>
 </sst>
 </file>
@@ -2427,8 +2430,8 @@
       <xdr:rowOff>8142</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1174617" cy="172227"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="TextBox 1">
@@ -2657,7 +2660,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="TextBox 1">
@@ -2752,8 +2755,8 @@
       <xdr:rowOff>17837</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="4494948" cy="172098"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="3" name="TextBox 2">
@@ -3375,7 +3378,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="3" name="TextBox 2">
@@ -3465,12 +3468,16 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{214BFB70-A220-7742-A104-C82532B69A95}" name="col_legend" displayName="col_legend" ref="A1:B34" totalsRowShown="0" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{214BFB70-A220-7742-A104-C82532B69A95}" name="col_legend" displayName="col_legend" ref="A1:B34" totalsRowShown="0" dataDxfId="2">
   <autoFilter ref="A1:B34" xr:uid="{214BFB70-A220-7742-A104-C82532B69A95}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{19BC19FB-B4CA-5F43-A4FD-BF2AC7E7A690}" name="columns" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{52C1B72F-FDFD-3C42-9813-D2D0A30F0F91}" name="description" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{19BC19FB-B4CA-5F43-A4FD-BF2AC7E7A690}" name="columns" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{52C1B72F-FDFD-3C42-9813-D2D0A30F0F91}" name="description" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight20" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -18851,7 +18858,7 @@
         <v>676</v>
       </c>
       <c r="C174" t="s">
-        <v>679</v>
+        <v>775</v>
       </c>
       <c r="D174" t="s">
         <v>42</v>

</xml_diff>